<commit_message>
fix: refresh telegram sebi verification metrics for 1-Sep audit
</commit_message>
<xml_diff>
--- a/data/non_sebi_creators_cumulative.xlsx
+++ b/data/non_sebi_creators_cumulative.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Non-SEBI Master Registry" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-SEBI Master Registry" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -569,7 +569,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Generated On: 2026-09-01 04:47:48 | Daily Audits Logged: 3</t>
+          <t>Generated On: 2026-09-01 10:33:03 | Daily Audits Logged: 3</t>
         </is>
       </c>
     </row>
@@ -680,10 +680,10 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0</v>
+        <v>393</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>0</v>
+        <v>4385088</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: enhance self-transaction detection, live product deliverable verification, and top-priority flags
</commit_message>
<xml_diff>
--- a/data/non_sebi_creators_cumulative.xlsx
+++ b/data/non_sebi_creators_cumulative.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Non-SEBI Master Registry" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-SEBI Master Registry" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -569,7 +569,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Generated On: 2026-09-12 06:22:16 | Daily Audits Logged: 14</t>
+          <t>Generated On: 2026-09-12 12:17:42 | Daily Audits Logged: 14</t>
         </is>
       </c>
     </row>

</xml_diff>